<commit_message>
feat: add Python script to automate generation and backup of the TOPSIM CFO dashboard Excel file
</commit_message>
<xml_diff>
--- a/TOPSIM_CFO_Dashboard.xlsx
+++ b/TOPSIM_CFO_Dashboard.xlsx
@@ -51,9 +51,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -694,7 +695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -767,163 +768,182 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>--- KERNAUSGABEN ---</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
+          <t>Geplante Produktionsmenge</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>45000</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Für Bestandsveränderung</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Total Herstellkosten</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>90</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>MEUR</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>inkl. Personal in Fertigung</t>
-        </is>
-      </c>
+          <t>--- FERTIGUNG &amp; PERSONAL (HERSTELLKOSTEN) ---</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Total Verwaltungskosten</t>
+          <t>Material- &amp; Maschinenkosten</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>MEUR</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Reine Sachkosten Fertigung</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Total Marketing/Vertrieb</t>
+          <t>Anzahl Fertigungsmitarbeiter</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>850</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MEUR</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
+          <t>Personen</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Geplanter Bestand</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Forschung &amp; Entwicklung (F&amp;E)</t>
+          <t>Ø Gehalt pro Mitarbeiter</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2.5</v>
+        <v>40000</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MEUR</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ökologie, Technologie, etc.</t>
+          <t>Basisgehalt (Aus Berichten ablesen)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Marktforschung</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0.15</v>
+          <t>Personalnebenkosten (%)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>0.4</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MEUR</t>
+          <t>%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Kosten für Berichte / Analysen</t>
+          <t>Normalerweise 40%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>--- INVESTITIONEN ---</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+          <t>Trainingsbudget pro MA</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1600</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Z.B. 1600 EUR</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Freiwillige Tilgung Langfristkr.</t>
+          <t>Anzahl Einstellungen/Entlassungen</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MEUR</t>
+          <t>Personen</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Cash-Out! Kurzfrist wird automatisch getilgt.</t>
+          <t>Fluktuation + aktive Wechsel</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Abschreibungen Alt-Anlagen</t>
+          <t>Kosten pro Wechsel</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6</v>
+        <v>5000</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MEUR</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>inklusive 0.25 MEUR fixe Gebäude-AfA</t>
+          <t>Recruiting-/Abfindungskosten</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Geplante Neuinvestition</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>15</v>
+          <t>Total Herstellkosten (Berechnet)</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>B6 + ((B7*B8*(1+B9) + B7*B10 + B11*B12)/1000000)</f>
+        <v/>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -932,67 +952,179 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Totaler Kaufpreis Anlage - Cash Out!</t>
+          <t>Fließt ins EBIT ein</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Geplante Neu-Abschreibung</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>MEUR</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Z.B. 10% Lineare Abschreibung</t>
-        </is>
-      </c>
+          <t>--- WEITERE OPERATIVE KOSTEN ---</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Veränderung Pensionsrückstellungen</t>
+          <t>Total Verwaltungskosten</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>MEUR</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Positiv = Cash-plus</t>
-        </is>
-      </c>
+      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Geplante Produktionsmenge</t>
+          <t>Total Marketing/Vertrieb</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>45000</v>
+        <v>15</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Stück</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Für Bestandsveränderung (Fertigung)</t>
+          <t>MEUR</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Forschung &amp; Entwicklung (F&amp;E)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MEUR</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Ökologie, Technologie, etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Marktforschung</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MEUR</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Kosten für Berichte / Analysen</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>--- INVESTITIONEN ---</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Abschreibungen Alt-Anlagen</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>6</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MEUR</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>inklusive 0.25 MEUR fixe Gebäude-AfA</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Geplante Neuinvestition</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>15</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MEUR</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Totaler Kaufpreis Anlage - Cash Out!</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Geplante Neu-Abschreibung</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MEUR</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Z.B. 10% Lineare Abschreibung</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Veränderung Pensionsrückstellungen</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MEUR</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Positiv = Cash-plus</t>
         </is>
       </c>
     </row>
@@ -1147,15 +1279,15 @@
         </is>
       </c>
       <c r="B9">
-        <f>IF('2_Team_Inputs'!B16&gt;0, ('2_Team_Inputs'!B16-'2_Team_Inputs'!B2)*('2_Team_Inputs'!B5/'2_Team_Inputs'!B16), 0)</f>
+        <f>IF('2_Team_Inputs'!B4&gt;0, ('2_Team_Inputs'!B4-'2_Team_Inputs'!B2)*('2_Team_Inputs'!B13/'2_Team_Inputs'!B4), 0)</f>
         <v/>
       </c>
       <c r="C9">
-        <f>IF('2_Team_Inputs'!B16&gt;0, ('2_Team_Inputs'!B16-'2_Team_Inputs'!B2)*('2_Team_Inputs'!B5/'2_Team_Inputs'!B16), 0)</f>
+        <f>IF('2_Team_Inputs'!B4&gt;0, ('2_Team_Inputs'!B4-'2_Team_Inputs'!B2)*('2_Team_Inputs'!B13/'2_Team_Inputs'!B4), 0)</f>
         <v/>
       </c>
       <c r="D9">
-        <f>IF('2_Team_Inputs'!B16&gt;0, ('2_Team_Inputs'!B16-'2_Team_Inputs'!B2)*('2_Team_Inputs'!B5/'2_Team_Inputs'!B16), 0)</f>
+        <f>IF('2_Team_Inputs'!B4&gt;0, ('2_Team_Inputs'!B4-'2_Team_Inputs'!B2)*('2_Team_Inputs'!B13/'2_Team_Inputs'!B4), 0)</f>
         <v/>
       </c>
     </row>
@@ -1166,15 +1298,15 @@
         </is>
       </c>
       <c r="B10">
-        <f>B8+B9-SUM('2_Team_Inputs'!B5:B9)-'2_Team_Inputs'!B12-'2_Team_Inputs'!B14</f>
+        <f>B8+B9-'2_Team_Inputs'!B13-SUM('2_Team_Inputs'!B15:B18)-'2_Team_Inputs'!B20-'2_Team_Inputs'!B22</f>
         <v/>
       </c>
       <c r="C10">
-        <f>C8+C9-SUM('2_Team_Inputs'!B5:B9)-'2_Team_Inputs'!B12-'2_Team_Inputs'!B14</f>
+        <f>C8+C9-'2_Team_Inputs'!B13-SUM('2_Team_Inputs'!B15:B18)-'2_Team_Inputs'!B20-'2_Team_Inputs'!B22</f>
         <v/>
       </c>
       <c r="D10">
-        <f>D8+D9-SUM('2_Team_Inputs'!B5:B9)-'2_Team_Inputs'!B12-'2_Team_Inputs'!B14</f>
+        <f>D8+D9-'2_Team_Inputs'!B13-SUM('2_Team_Inputs'!B15:B18)-'2_Team_Inputs'!B20-'2_Team_Inputs'!B22</f>
         <v/>
       </c>
     </row>
@@ -1185,15 +1317,15 @@
         </is>
       </c>
       <c r="B11">
-        <f>((B3+'1_Ist_Daten'!B7)*'1_Ist_Daten'!B11)+((B4+'1_Ist_Daten'!B8-'2_Team_Inputs'!B11)*'1_Ist_Daten'!B10)</f>
+        <f>((B3+'1_Ist_Daten'!B7)*'1_Ist_Daten'!B11)+((B4+'1_Ist_Daten'!B8)*'1_Ist_Daten'!B10)</f>
         <v/>
       </c>
       <c r="C11">
-        <f>((C3+'1_Ist_Daten'!B7)*'1_Ist_Daten'!B11)+((C4+'1_Ist_Daten'!B8-'2_Team_Inputs'!B11)*'1_Ist_Daten'!B10)</f>
+        <f>((C3+'1_Ist_Daten'!B7)*'1_Ist_Daten'!B11)+((C4+'1_Ist_Daten'!B8)*'1_Ist_Daten'!B10)</f>
         <v/>
       </c>
       <c r="D11">
-        <f>((D3+'1_Ist_Daten'!B7)*'1_Ist_Daten'!B11)+((D4+'1_Ist_Daten'!B8-'2_Team_Inputs'!B11)*'1_Ist_Daten'!B10)</f>
+        <f>((D3+'1_Ist_Daten'!B7)*'1_Ist_Daten'!B11)+((D4+'1_Ist_Daten'!B8)*'1_Ist_Daten'!B10)</f>
         <v/>
       </c>
     </row>
@@ -1328,15 +1460,15 @@
         </is>
       </c>
       <c r="B19">
-        <f>B15+'2_Team_Inputs'!B12+'2_Team_Inputs'!B14+'2_Team_Inputs'!B15</f>
+        <f>B15+'2_Team_Inputs'!B20+'2_Team_Inputs'!B22+'2_Team_Inputs'!B23</f>
         <v/>
       </c>
       <c r="C19">
-        <f>C15+'2_Team_Inputs'!B12+'2_Team_Inputs'!B14+'2_Team_Inputs'!B15</f>
+        <f>C15+'2_Team_Inputs'!B20+'2_Team_Inputs'!B22+'2_Team_Inputs'!B23</f>
         <v/>
       </c>
       <c r="D19">
-        <f>D15+'2_Team_Inputs'!B12+'2_Team_Inputs'!B14+'2_Team_Inputs'!B15</f>
+        <f>D15+'2_Team_Inputs'!B20+'2_Team_Inputs'!B22+'2_Team_Inputs'!B23</f>
         <v/>
       </c>
     </row>
@@ -1357,15 +1489,15 @@
         </is>
       </c>
       <c r="B21">
-        <f>'1_Ist_Daten'!B2+B19+B3+B4-B5-'2_Team_Inputs'!B13-'1_Ist_Daten'!B7-'2_Team_Inputs'!B11-B6</f>
+        <f>'1_Ist_Daten'!B2+B19+B3+B4-B5-B6-'2_Team_Inputs'!B21-'1_Ist_Daten'!B7</f>
         <v/>
       </c>
       <c r="C21">
-        <f>'1_Ist_Daten'!B2+C19+C3+C4-C5-'2_Team_Inputs'!B13-'1_Ist_Daten'!B7-'2_Team_Inputs'!B11-C6</f>
+        <f>'1_Ist_Daten'!B2+C19+C3+C4-C5-C6-'2_Team_Inputs'!B21-'1_Ist_Daten'!B7</f>
         <v/>
       </c>
       <c r="D21">
-        <f>'1_Ist_Daten'!B2+D19+D3+D4-D5-'2_Team_Inputs'!B13-'1_Ist_Daten'!B7-'2_Team_Inputs'!B11-D6</f>
+        <f>'1_Ist_Daten'!B2+D19+D3+D4-D5-D6-'2_Team_Inputs'!B21-'1_Ist_Daten'!B7</f>
         <v/>
       </c>
     </row>

</xml_diff>